<commit_message>
Read invoice PDFs from Gmail inbox (IMAP) instead of local text files
- gmail_ingest.py: pull PDF attachments over IMAP (App Password) + extract text with pypdf
- generate_sample_pdfs.py: render mock invoices to PDFs for emailing/testing
- extract.py: accept invoice sources (Gmail PDFs or local .txt fallback)
- main.py: ingest step chooses source via INVOICE_SOURCE (default gmail)
- is_invoice guard: LLM flags non-invoice PDFs; pipeline skips them
- Docs + diagram updated; sample_output captured from a real Gmail run
</commit_message>
<xml_diff>
--- a/sample_output/invoice_tracker.xlsx
+++ b/sample_output/invoice_tracker.xlsx
@@ -473,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,7 +511,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -549,7 +549,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-13 02:18</t>
+          <t>2026-06-16 21:44</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">

</xml_diff>